<commit_message>
add asda mobile to the service
</commit_message>
<xml_diff>
--- a/public/collecting-mobile-information/extra-mobile-data-requests-template.xlsx
+++ b/public/collecting-mobile-information/extra-mobile-data-requests-template.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="25">
   <si>
     <t xml:space="preserve">Account holder name</t>
   </si>
@@ -53,6 +53,9 @@
   </si>
   <si>
     <t xml:space="preserve">Mobile networks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asda Mobile</t>
   </si>
   <si>
     <t xml:space="preserve">BT Mobile</t>
@@ -345,12 +348,12 @@
       <formula1>"TRUE,FALSE"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C3:C10" type="list">
-      <formula1>",BT Mobile,EE,Lycamobile,O2,Sky Mobile,SMARTY,Tesco Mobile,Three,Virgin Mobile,Vodafone,iD Mobile"</formula1>
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C2" type="list">
+      <formula1>"Asda Mobile,BT Mobile,EE,giffgaff,Lycamobile,O2,Sky Mobile,SMARTY,Tesco Mobile,Three,Virgin Mobile,Vodafone,iD Mobile"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C2" type="list">
-      <formula1>"BT Mobile,EE,giffgaff,Lycamobile,O2,Sky Mobile,SMARTY,Tesco Mobile,Three,Virgin Mobile,Vodafone,iD Mobile"</formula1>
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C3:C10" type="list">
+      <formula1>",Asda Mobile,BT Mobile,EE,Lycamobile,O2,Sky Mobile,SMARTY,Tesco Mobile,Three,Virgin Mobile,Vodafone,iD Mobile"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -369,7 +372,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultColWidth="10.859375" defaultRowHeight="16" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.35"/>
@@ -405,7 +408,7 @@
     </row>
     <row r="4" customFormat="false" ht="15.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -414,7 +417,7 @@
     </row>
     <row r="5" customFormat="false" ht="15.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -492,6 +495,15 @@
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
+    </row>
+    <row r="14" customFormat="false" ht="15.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -518,7 +530,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -527,7 +539,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -617,7 +629,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>

</xml_diff>